<commit_message>
feat(marketing): aggiornato copy booking diretto con split 50/50
</commit_message>
<xml_diff>
--- a/documenti/VirtualBNB-Modello-Finanziario.xlsx
+++ b/documenti/VirtualBNB-Modello-Finanziario.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="102">
   <si>
     <t xml:space="preserve">VirtualBNB — Assunzioni del Modello</t>
   </si>
@@ -122,6 +122,36 @@
     <t xml:space="preserve">SOSTITUISCI col numero vero — decide quante proprietà ti servono davvero</t>
   </si>
   <si>
+    <t xml:space="preserve">Prenotazioni dirette — risparmio netto reale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commissione OTA evitata (stima, lorda)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Media indicativa del range 15-17% dichiarato in Servizi.jsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fee Lodgify su prenotazione diretta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Piani Starter/Professional. Diventa 0% sul piano Ultimate — verifica quale piano hai scelto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risparmio netto reale (% da dividere con il proprietario)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Esempio su una prenotazione diretta di:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risparmio lordo (commissione OTA evitata)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meno: fee Lodgify sulla prenotazione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risparmio netto da dividere con il proprietario</t>
+  </si>
+  <si>
     <t xml:space="preserve">Costi Fissi Mensili — indipendenti dal numero di immobili</t>
   </si>
   <si>
@@ -174,6 +204,12 @@
   </si>
   <si>
     <t xml:space="preserve">STIMA — verifica polizza reale, valutane la necessità</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lodgify (Professional — channel manager + booking diretto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STIMA — dipende dal piano scelto (Starter/Professional/Ultimate) e dal numero di immobili collegati, verifica col tuo account reale</t>
   </si>
   <si>
     <t xml:space="preserve">TOTALE COSTI FISSI MENSILI</t>
@@ -475,20 +511,24 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="40">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -500,51 +540,59 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -552,47 +600,75 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -848,202 +924,273 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="50"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5" t="s">
+      <c r="C5" s="6"/>
+      <c r="D5" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="8" t="n">
         <v>0.25</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="7" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="8" t="n">
         <v>0.28</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="9" t="n">
         <v>650</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="7" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="8" t="n">
+      <c r="B11" s="9" t="n">
         <v>350</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="8" t="n">
+      <c r="B12" s="9" t="n">
         <v>450</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="8" t="n">
+      <c r="B13" s="9" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="10" t="n">
+      <c r="B15" s="11" t="n">
         <f aca="false">B8/B7</f>
         <v>2321.42857142857</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5" t="s">
+      <c r="C18" s="6"/>
+      <c r="D18" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="11" t="n">
+      <c r="B19" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D19" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="12" t="n">
+      <c r="B20" s="13" t="n">
         <v>22</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="D20" s="7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="11" t="n">
+      <c r="B21" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="D21" s="7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B22" s="13" t="n">
+      <c r="B22" s="14" t="n">
         <v>0.5</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="D22" s="7" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="9" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="14" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="15" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="15" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="16" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="9" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="10" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="6" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B29" s="16" t="n">
+      <c r="B29" s="17" t="n">
         <v>2000</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="D29" s="7" t="s">
         <v>31</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="18" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B32" s="19" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="D32" s="20" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" s="19" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="D33" s="20" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="B34" s="22" t="n">
+        <f aca="false">B32-B33</f>
+        <v>0.141</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B36" s="23" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C37" s="24" t="n">
+        <f aca="false">B36*B32</f>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C38" s="24" t="n">
+        <f aca="false">B36*B33</f>
+        <v>2.85</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="C39" s="25" t="n">
+        <f aca="false">C37-C38</f>
+        <v>21.15</v>
       </c>
     </row>
   </sheetData>
@@ -1065,127 +1212,138 @@
   <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="50"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C4" s="5" t="s">
+      <c r="B4" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B5" s="11" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="12" t="n">
         <v>20</v>
       </c>
-      <c r="C5" s="17" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B6" s="11" t="n">
+      <c r="C5" s="26" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" s="12" t="n">
         <v>25</v>
       </c>
-      <c r="C6" s="17" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B7" s="11" t="n">
+      <c r="C6" s="26" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="26" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="C8" s="26" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C9" s="26" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="26" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="C11" s="26" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12" s="13" t="n">
         <v>40</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="B8" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="C8" s="17" t="s">
+      <c r="C12" s="26" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B13" s="27" t="n">
         <v>42</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B9" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="C9" s="17" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B10" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B11" s="12" t="n">
-        <v>100</v>
-      </c>
-      <c r="C11" s="17" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="B12" s="12" t="n">
-        <v>40</v>
-      </c>
-      <c r="C12" s="17" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="B14" s="19" t="n">
+      <c r="C13" s="20" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="28" t="s">
+        <v>62</v>
+      </c>
+      <c r="B14" s="29" t="n">
         <f aca="false">SUM(B5:B13)</f>
-        <v>211</v>
+        <v>253</v>
       </c>
     </row>
   </sheetData>
@@ -1207,367 +1365,367 @@
   <dimension ref="A1:D33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="1" width="16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
-        <v>51</v>
-      </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4"/>
-      <c r="B4" s="5" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5"/>
+      <c r="B4" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="B5" s="11" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B5" s="12" t="n">
         <v>850</v>
       </c>
-      <c r="C5" s="11" t="n">
+      <c r="C5" s="12" t="n">
         <v>850</v>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D5" s="12" t="n">
         <v>850</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B6" s="21" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="B6" s="31" t="n">
         <f aca="false">B5*Assunzioni!$B$6</f>
         <v>212.5</v>
       </c>
-      <c r="C6" s="21" t="n">
+      <c r="C6" s="31" t="n">
         <f aca="false">C5*Assunzioni!$B$7</f>
         <v>238</v>
       </c>
-      <c r="D6" s="21" t="n">
+      <c r="D6" s="31" t="n">
         <f aca="false">Assunzioni!$B$8</f>
         <v>650</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
-        <v>55</v>
-      </c>
-      <c r="B7" s="19" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="B7" s="29" t="n">
         <f aca="false">B5-B6</f>
         <v>637.5</v>
       </c>
-      <c r="C7" s="19" t="n">
+      <c r="C7" s="29" t="n">
         <f aca="false">C5-C6</f>
         <v>612</v>
       </c>
-      <c r="D7" s="19" t="n">
+      <c r="D7" s="29" t="n">
         <f aca="false">D5-D6</f>
         <v>200</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B8" s="21" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B8" s="31" t="n">
         <f aca="false">Assunzioni!$B$19+Assunzioni!$B$20</f>
         <v>24</v>
       </c>
-      <c r="C8" s="21" t="n">
+      <c r="C8" s="31" t="n">
         <f aca="false">Assunzioni!$B$19+Assunzioni!$B$20</f>
         <v>24</v>
       </c>
-      <c r="D8" s="21" t="n">
+      <c r="D8" s="31" t="n">
         <f aca="false">Assunzioni!$B$19+Assunzioni!$B$20</f>
         <v>24</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B9" s="23" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="21" t="n">
+      <c r="C9" s="31" t="n">
         <f aca="false">Assunzioni!$B$21*Assunzioni!$B$22</f>
         <v>50</v>
       </c>
-      <c r="D9" s="23" t="n">
+      <c r="D9" s="33" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="22" t="s">
-        <v>58</v>
-      </c>
-      <c r="B10" s="19" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="32" t="s">
+        <v>70</v>
+      </c>
+      <c r="B10" s="29" t="n">
         <f aca="false">B6-B8-B9</f>
         <v>188.5</v>
       </c>
-      <c r="C10" s="19" t="n">
+      <c r="C10" s="29" t="n">
         <f aca="false">C6-C8-C9</f>
         <v>164</v>
       </c>
-      <c r="D10" s="19" t="n">
+      <c r="D10" s="29" t="n">
         <f aca="false">D6-D8-D9</f>
         <v>626</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4"/>
-      <c r="B14" s="5" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5"/>
+      <c r="B14" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="B15" s="11" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B15" s="12" t="n">
         <v>2120</v>
       </c>
-      <c r="C15" s="11" t="n">
+      <c r="C15" s="12" t="n">
         <v>2120</v>
       </c>
-      <c r="D15" s="11" t="n">
+      <c r="D15" s="12" t="n">
         <v>2120</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B16" s="21" t="n">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="B16" s="31" t="n">
         <f aca="false">B15*Assunzioni!$B$6</f>
         <v>530</v>
       </c>
-      <c r="C16" s="21" t="n">
+      <c r="C16" s="31" t="n">
         <f aca="false">C15*Assunzioni!$B$7</f>
         <v>593.6</v>
       </c>
-      <c r="D16" s="21" t="n">
+      <c r="D16" s="31" t="n">
         <f aca="false">Assunzioni!$B$8</f>
         <v>650</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="22" t="s">
-        <v>55</v>
-      </c>
-      <c r="B17" s="19" t="n">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="B17" s="29" t="n">
         <f aca="false">B15-B16</f>
         <v>1590</v>
       </c>
-      <c r="C17" s="19" t="n">
+      <c r="C17" s="29" t="n">
         <f aca="false">C15-C16</f>
         <v>1526.4</v>
       </c>
-      <c r="D17" s="19" t="n">
+      <c r="D17" s="29" t="n">
         <f aca="false">D15-D16</f>
         <v>1470</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B18" s="21" t="n">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B18" s="31" t="n">
         <f aca="false">Assunzioni!$B$19+Assunzioni!$B$20</f>
         <v>24</v>
       </c>
-      <c r="C18" s="21" t="n">
+      <c r="C18" s="31" t="n">
         <f aca="false">Assunzioni!$B$19+Assunzioni!$B$20</f>
         <v>24</v>
       </c>
-      <c r="D18" s="21" t="n">
+      <c r="D18" s="31" t="n">
         <f aca="false">Assunzioni!$B$19+Assunzioni!$B$20</f>
         <v>24</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B19" s="23" t="n">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B19" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="C19" s="21" t="n">
+      <c r="C19" s="31" t="n">
         <f aca="false">Assunzioni!$B$21*Assunzioni!$B$22</f>
         <v>50</v>
       </c>
-      <c r="D19" s="23" t="n">
+      <c r="D19" s="33" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="22" t="s">
-        <v>58</v>
-      </c>
-      <c r="B20" s="19" t="n">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="32" t="s">
+        <v>70</v>
+      </c>
+      <c r="B20" s="29" t="n">
         <f aca="false">B16-B18-B19</f>
         <v>506</v>
       </c>
-      <c r="C20" s="19" t="n">
+      <c r="C20" s="29" t="n">
         <f aca="false">C16-C18-C19</f>
         <v>519.6</v>
       </c>
-      <c r="D20" s="19" t="n">
+      <c r="D20" s="29" t="n">
         <f aca="false">D16-D18-D19</f>
         <v>626</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4"/>
-      <c r="B24" s="5" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5"/>
+      <c r="B24" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="D24" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="B25" s="11" t="n">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B25" s="12" t="n">
         <v>3510</v>
       </c>
-      <c r="C25" s="11" t="n">
+      <c r="C25" s="12" t="n">
         <v>3510</v>
       </c>
-      <c r="D25" s="11" t="n">
+      <c r="D25" s="12" t="n">
         <v>3510</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B26" s="21" t="n">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="B26" s="31" t="n">
         <f aca="false">B25*Assunzioni!$B$6</f>
         <v>877.5</v>
       </c>
-      <c r="C26" s="21" t="n">
+      <c r="C26" s="31" t="n">
         <f aca="false">C25*Assunzioni!$B$7</f>
         <v>982.8</v>
       </c>
-      <c r="D26" s="21" t="n">
+      <c r="D26" s="31" t="n">
         <f aca="false">Assunzioni!$B$8</f>
         <v>650</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="22" t="s">
-        <v>55</v>
-      </c>
-      <c r="B27" s="19" t="n">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="B27" s="29" t="n">
         <f aca="false">B25-B26</f>
         <v>2632.5</v>
       </c>
-      <c r="C27" s="19" t="n">
+      <c r="C27" s="29" t="n">
         <f aca="false">C25-C26</f>
         <v>2527.2</v>
       </c>
-      <c r="D27" s="19" t="n">
+      <c r="D27" s="29" t="n">
         <f aca="false">D25-D26</f>
         <v>2860</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B28" s="21" t="n">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B28" s="31" t="n">
         <f aca="false">Assunzioni!$B$19+Assunzioni!$B$20</f>
         <v>24</v>
       </c>
-      <c r="C28" s="21" t="n">
+      <c r="C28" s="31" t="n">
         <f aca="false">Assunzioni!$B$19+Assunzioni!$B$20</f>
         <v>24</v>
       </c>
-      <c r="D28" s="21" t="n">
+      <c r="D28" s="31" t="n">
         <f aca="false">Assunzioni!$B$19+Assunzioni!$B$20</f>
         <v>24</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B29" s="23" t="n">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B29" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="C29" s="21" t="n">
+      <c r="C29" s="31" t="n">
         <f aca="false">Assunzioni!$B$21*Assunzioni!$B$22</f>
         <v>50</v>
       </c>
-      <c r="D29" s="23" t="n">
+      <c r="D29" s="33" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="22" t="s">
-        <v>58</v>
-      </c>
-      <c r="B30" s="19" t="n">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="32" t="s">
+        <v>70</v>
+      </c>
+      <c r="B30" s="29" t="n">
         <f aca="false">B26-B28-B29</f>
         <v>853.5</v>
       </c>
-      <c r="C30" s="19" t="n">
+      <c r="C30" s="29" t="n">
         <f aca="false">C26-C28-C29</f>
         <v>908.8</v>
       </c>
-      <c r="D30" s="19" t="n">
+      <c r="D30" s="29" t="n">
         <f aca="false">D26-D28-D29</f>
         <v>626</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="B33" s="24"/>
-      <c r="C33" s="24"/>
-      <c r="D33" s="24"/>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="34" t="s">
+        <v>73</v>
+      </c>
+      <c r="B33" s="34"/>
+      <c r="C33" s="34"/>
+      <c r="D33" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1592,60 +1750,60 @@
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="50"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="B3" s="21" t="n">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B3" s="31" t="n">
         <f aca="false">'Costi Fissi Azienda'!B14</f>
-        <v>211</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="B4" s="21" t="n">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="B4" s="31" t="n">
         <f aca="false">Assunzioni!B29</f>
         <v>2000</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="B5" s="19" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B5" s="29" t="n">
         <f aca="false">B3+B4</f>
-        <v>2211</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="B7" s="21" t="n">
+        <v>2253</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B7" s="31" t="n">
         <f aca="false">'P&amp;L per Tier'!C20</f>
         <v>519.6</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="22" t="s">
-        <v>68</v>
-      </c>
-      <c r="B9" s="25" t="n">
+      <c r="C7" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="B9" s="35" t="n">
         <f aca="false">ROUNDUP(B5/B7,0)</f>
         <v>5</v>
       </c>
@@ -1669,390 +1827,390 @@
   <dimension ref="A1:M11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="2" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="2" style="1" width="9"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="L3" s="5" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="30" t="s">
         <v>81</v>
       </c>
-      <c r="M3" s="5" t="s">
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
+      <c r="M1" s="30"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
+      <c r="B3" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="B4" s="26" t="n">
+      <c r="C3" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="B4" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="26" t="n">
+      <c r="C4" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="26" t="n">
+      <c r="D4" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="26" t="n">
+      <c r="E4" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="F4" s="26" t="n">
+      <c r="F4" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="26" t="n">
+      <c r="G4" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="H4" s="26" t="n">
+      <c r="H4" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="I4" s="26" t="n">
+      <c r="I4" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="J4" s="26" t="n">
+      <c r="J4" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="K4" s="26" t="n">
+      <c r="K4" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="L4" s="26" t="n">
+      <c r="L4" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="M4" s="26" t="n">
+      <c r="M4" s="36" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="B5" s="27" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B5" s="37" t="n">
         <f aca="false">B4</f>
         <v>1</v>
       </c>
-      <c r="C5" s="27" t="n">
+      <c r="C5" s="37" t="n">
         <f aca="false">B5+C4</f>
         <v>2</v>
       </c>
-      <c r="D5" s="27" t="n">
+      <c r="D5" s="37" t="n">
         <f aca="false">C5+D4</f>
         <v>3</v>
       </c>
-      <c r="E5" s="27" t="n">
+      <c r="E5" s="37" t="n">
         <f aca="false">D5+E4</f>
         <v>4</v>
       </c>
-      <c r="F5" s="27" t="n">
+      <c r="F5" s="37" t="n">
         <f aca="false">E5+F4</f>
         <v>5</v>
       </c>
-      <c r="G5" s="27" t="n">
+      <c r="G5" s="37" t="n">
         <f aca="false">F5+G4</f>
         <v>6</v>
       </c>
-      <c r="H5" s="27" t="n">
+      <c r="H5" s="37" t="n">
         <f aca="false">G5+H4</f>
         <v>7</v>
       </c>
-      <c r="I5" s="27" t="n">
+      <c r="I5" s="37" t="n">
         <f aca="false">H5+I4</f>
         <v>8</v>
       </c>
-      <c r="J5" s="27" t="n">
+      <c r="J5" s="37" t="n">
         <f aca="false">I5+J4</f>
         <v>9</v>
       </c>
-      <c r="K5" s="27" t="n">
+      <c r="K5" s="37" t="n">
         <f aca="false">J5+K4</f>
         <v>10</v>
       </c>
-      <c r="L5" s="27" t="n">
+      <c r="L5" s="37" t="n">
         <f aca="false">K5+L4</f>
         <v>11</v>
       </c>
-      <c r="M5" s="27" t="n">
+      <c r="M5" s="37" t="n">
         <f aca="false">L5+M4</f>
         <v>12</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="B6" s="28" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="B6" s="38" t="n">
         <f aca="false">B5*Breakeven!$B$7</f>
         <v>519.6</v>
       </c>
-      <c r="C6" s="28" t="n">
+      <c r="C6" s="38" t="n">
         <f aca="false">C5*Breakeven!$B$7</f>
         <v>1039.2</v>
       </c>
-      <c r="D6" s="28" t="n">
+      <c r="D6" s="38" t="n">
         <f aca="false">D5*Breakeven!$B$7</f>
         <v>1558.8</v>
       </c>
-      <c r="E6" s="28" t="n">
+      <c r="E6" s="38" t="n">
         <f aca="false">E5*Breakeven!$B$7</f>
         <v>2078.4</v>
       </c>
-      <c r="F6" s="28" t="n">
+      <c r="F6" s="38" t="n">
         <f aca="false">F5*Breakeven!$B$7</f>
         <v>2598</v>
       </c>
-      <c r="G6" s="28" t="n">
+      <c r="G6" s="38" t="n">
         <f aca="false">G5*Breakeven!$B$7</f>
         <v>3117.6</v>
       </c>
-      <c r="H6" s="28" t="n">
+      <c r="H6" s="38" t="n">
         <f aca="false">H5*Breakeven!$B$7</f>
         <v>3637.2</v>
       </c>
-      <c r="I6" s="28" t="n">
+      <c r="I6" s="38" t="n">
         <f aca="false">I5*Breakeven!$B$7</f>
         <v>4156.8</v>
       </c>
-      <c r="J6" s="28" t="n">
+      <c r="J6" s="38" t="n">
         <f aca="false">J5*Breakeven!$B$7</f>
         <v>4676.4</v>
       </c>
-      <c r="K6" s="28" t="n">
+      <c r="K6" s="38" t="n">
         <f aca="false">K5*Breakeven!$B$7</f>
         <v>5196</v>
       </c>
-      <c r="L6" s="28" t="n">
+      <c r="L6" s="38" t="n">
         <f aca="false">L5*Breakeven!$B$7</f>
         <v>5715.6</v>
       </c>
-      <c r="M6" s="28" t="n">
+      <c r="M6" s="38" t="n">
         <f aca="false">M5*Breakeven!$B$7</f>
         <v>6235.2</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="B7" s="28" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="B7" s="38" t="n">
         <f aca="false">'Costi Fissi Azienda'!$B$14</f>
-        <v>211</v>
-      </c>
-      <c r="C7" s="28" t="n">
+        <v>253</v>
+      </c>
+      <c r="C7" s="38" t="n">
         <f aca="false">'Costi Fissi Azienda'!$B$14</f>
-        <v>211</v>
-      </c>
-      <c r="D7" s="28" t="n">
+        <v>253</v>
+      </c>
+      <c r="D7" s="38" t="n">
         <f aca="false">'Costi Fissi Azienda'!$B$14</f>
-        <v>211</v>
-      </c>
-      <c r="E7" s="28" t="n">
+        <v>253</v>
+      </c>
+      <c r="E7" s="38" t="n">
         <f aca="false">'Costi Fissi Azienda'!$B$14</f>
-        <v>211</v>
-      </c>
-      <c r="F7" s="28" t="n">
+        <v>253</v>
+      </c>
+      <c r="F7" s="38" t="n">
         <f aca="false">'Costi Fissi Azienda'!$B$14</f>
-        <v>211</v>
-      </c>
-      <c r="G7" s="28" t="n">
+        <v>253</v>
+      </c>
+      <c r="G7" s="38" t="n">
         <f aca="false">'Costi Fissi Azienda'!$B$14</f>
-        <v>211</v>
-      </c>
-      <c r="H7" s="28" t="n">
+        <v>253</v>
+      </c>
+      <c r="H7" s="38" t="n">
         <f aca="false">'Costi Fissi Azienda'!$B$14</f>
-        <v>211</v>
-      </c>
-      <c r="I7" s="28" t="n">
+        <v>253</v>
+      </c>
+      <c r="I7" s="38" t="n">
         <f aca="false">'Costi Fissi Azienda'!$B$14</f>
-        <v>211</v>
-      </c>
-      <c r="J7" s="28" t="n">
+        <v>253</v>
+      </c>
+      <c r="J7" s="38" t="n">
         <f aca="false">'Costi Fissi Azienda'!$B$14</f>
-        <v>211</v>
-      </c>
-      <c r="K7" s="28" t="n">
+        <v>253</v>
+      </c>
+      <c r="K7" s="38" t="n">
         <f aca="false">'Costi Fissi Azienda'!$B$14</f>
-        <v>211</v>
-      </c>
-      <c r="L7" s="28" t="n">
+        <v>253</v>
+      </c>
+      <c r="L7" s="38" t="n">
         <f aca="false">'Costi Fissi Azienda'!$B$14</f>
-        <v>211</v>
-      </c>
-      <c r="M7" s="28" t="n">
+        <v>253</v>
+      </c>
+      <c r="M7" s="38" t="n">
         <f aca="false">'Costi Fissi Azienda'!$B$14</f>
-        <v>211</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="22" t="s">
-        <v>87</v>
-      </c>
-      <c r="B8" s="29" t="n">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="32" t="s">
+        <v>99</v>
+      </c>
+      <c r="B8" s="39" t="n">
         <f aca="false">B6-B7</f>
-        <v>308.6</v>
-      </c>
-      <c r="C8" s="29" t="n">
+        <v>266.6</v>
+      </c>
+      <c r="C8" s="39" t="n">
         <f aca="false">C6-C7</f>
-        <v>828.2</v>
-      </c>
-      <c r="D8" s="29" t="n">
+        <v>786.2</v>
+      </c>
+      <c r="D8" s="39" t="n">
         <f aca="false">D6-D7</f>
-        <v>1347.8</v>
-      </c>
-      <c r="E8" s="29" t="n">
+        <v>1305.8</v>
+      </c>
+      <c r="E8" s="39" t="n">
         <f aca="false">E6-E7</f>
-        <v>1867.4</v>
-      </c>
-      <c r="F8" s="29" t="n">
+        <v>1825.4</v>
+      </c>
+      <c r="F8" s="39" t="n">
         <f aca="false">F6-F7</f>
-        <v>2387</v>
-      </c>
-      <c r="G8" s="29" t="n">
+        <v>2345</v>
+      </c>
+      <c r="G8" s="39" t="n">
         <f aca="false">G6-G7</f>
-        <v>2906.6</v>
-      </c>
-      <c r="H8" s="29" t="n">
+        <v>2864.6</v>
+      </c>
+      <c r="H8" s="39" t="n">
         <f aca="false">H6-H7</f>
-        <v>3426.2</v>
-      </c>
-      <c r="I8" s="29" t="n">
+        <v>3384.2</v>
+      </c>
+      <c r="I8" s="39" t="n">
         <f aca="false">I6-I7</f>
-        <v>3945.8</v>
-      </c>
-      <c r="J8" s="29" t="n">
+        <v>3903.8</v>
+      </c>
+      <c r="J8" s="39" t="n">
         <f aca="false">J6-J7</f>
-        <v>4465.4</v>
-      </c>
-      <c r="K8" s="29" t="n">
+        <v>4423.4</v>
+      </c>
+      <c r="K8" s="39" t="n">
         <f aca="false">K6-K7</f>
-        <v>4985</v>
-      </c>
-      <c r="L8" s="29" t="n">
+        <v>4943</v>
+      </c>
+      <c r="L8" s="39" t="n">
         <f aca="false">L6-L7</f>
-        <v>5504.6</v>
-      </c>
-      <c r="M8" s="29" t="n">
+        <v>5462.6</v>
+      </c>
+      <c r="M8" s="39" t="n">
         <f aca="false">M6-M7</f>
-        <v>6024.2</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="22" t="s">
-        <v>88</v>
-      </c>
-      <c r="B9" s="29" t="n">
+        <v>5982.2</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="B9" s="39" t="n">
         <f aca="false">B8</f>
-        <v>308.6</v>
-      </c>
-      <c r="C9" s="29" t="n">
+        <v>266.6</v>
+      </c>
+      <c r="C9" s="39" t="n">
         <f aca="false">B9+C8</f>
-        <v>1136.8</v>
-      </c>
-      <c r="D9" s="29" t="n">
+        <v>1052.8</v>
+      </c>
+      <c r="D9" s="39" t="n">
         <f aca="false">C9+D8</f>
-        <v>2484.6</v>
-      </c>
-      <c r="E9" s="29" t="n">
+        <v>2358.6</v>
+      </c>
+      <c r="E9" s="39" t="n">
         <f aca="false">D9+E8</f>
-        <v>4352</v>
-      </c>
-      <c r="F9" s="29" t="n">
+        <v>4184</v>
+      </c>
+      <c r="F9" s="39" t="n">
         <f aca="false">E9+F8</f>
-        <v>6739</v>
-      </c>
-      <c r="G9" s="29" t="n">
+        <v>6529</v>
+      </c>
+      <c r="G9" s="39" t="n">
         <f aca="false">F9+G8</f>
-        <v>9645.6</v>
-      </c>
-      <c r="H9" s="29" t="n">
+        <v>9393.6</v>
+      </c>
+      <c r="H9" s="39" t="n">
         <f aca="false">G9+H8</f>
-        <v>13071.8</v>
-      </c>
-      <c r="I9" s="29" t="n">
+        <v>12777.8</v>
+      </c>
+      <c r="I9" s="39" t="n">
         <f aca="false">H9+I8</f>
-        <v>17017.6</v>
-      </c>
-      <c r="J9" s="29" t="n">
+        <v>16681.6</v>
+      </c>
+      <c r="J9" s="39" t="n">
         <f aca="false">I9+J8</f>
-        <v>21483</v>
-      </c>
-      <c r="K9" s="29" t="n">
+        <v>21105</v>
+      </c>
+      <c r="K9" s="39" t="n">
         <f aca="false">J9+K8</f>
-        <v>26468</v>
-      </c>
-      <c r="L9" s="29" t="n">
+        <v>26048</v>
+      </c>
+      <c r="L9" s="39" t="n">
         <f aca="false">K9+L8</f>
-        <v>31972.6</v>
-      </c>
-      <c r="M9" s="29" t="n">
+        <v>31510.6</v>
+      </c>
+      <c r="M9" s="39" t="n">
         <f aca="false">L9+M8</f>
-        <v>37996.8</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="24" t="s">
-        <v>89</v>
-      </c>
-      <c r="B11" s="24"/>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="24"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="24"/>
-      <c r="H11" s="24"/>
-      <c r="I11" s="24"/>
-      <c r="J11" s="24"/>
-      <c r="K11" s="24"/>
-      <c r="L11" s="24"/>
-      <c r="M11" s="24"/>
+        <v>37492.8</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="34" t="s">
+        <v>101</v>
+      </c>
+      <c r="B11" s="34"/>
+      <c r="C11" s="34"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="34"/>
+      <c r="F11" s="34"/>
+      <c r="G11" s="34"/>
+      <c r="H11" s="34"/>
+      <c r="I11" s="34"/>
+      <c r="J11" s="34"/>
+      <c r="K11" s="34"/>
+      <c r="L11" s="34"/>
+      <c r="M11" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>